<commit_message>
Changed fn.rownum in ID code bindings to return integer (instead of string)
</commit_message>
<xml_diff>
--- a/data/odm_v2/odm_v1_to_v2_id_code.xlsx
+++ b/data/odm_v2/odm_v1_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/odm_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE5A156-08DC-4349-ADE0-35F760199E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86E5C84F-561A-E947-B2F3-0A7AD8380CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -94,7 +94,7 @@
     <t>stepID</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.protocolSteps.measure[-3:] if datEmpty.protocolSteps.measure else datEmpty.protocolSteps.method[-3:])</t>
+    <t>fn.makeid(datEmpty.protocolSteps.measure[-3:] if datEmpty.protocolSteps.measure else datEmpty.protocolSteps.method[-3:], f"{fn.rownum:03d}")</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
ID generation code for all primary keys
</commit_message>
<xml_diff>
--- a/data/odm_v2/odm_v1_to_v2_id_code.xlsx
+++ b/data/odm_v2/odm_v1_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/odm_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AFDCD4B-2184-F746-9CFD-E7A15F3A92D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE629A60-1A16-E541-B1FF-BBCAA21A3C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>measures</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>fn.makeid(datEmpty.qualityReports.qualityFlag, datEmpty.qualityReports.measureRepID if datEmpty.qualityReports.__measureRepID else datEmpty.qualityReports.sampleID if datEmpty.qualityReports.__sampleID else datEmpty.qualityReports.measureSetRepID)</t>
-  </si>
-  <si>
-    <t>dat.measures.__measureRepID</t>
   </si>
   <si>
     <t>dat.measures.measureRepID</t>
@@ -102,6 +99,66 @@
   </si>
   <si>
     <t>dat.measures.__organizationID</t>
+  </si>
+  <si>
+    <t>contacts</t>
+  </si>
+  <si>
+    <t>instruments</t>
+  </si>
+  <si>
+    <t>organizations</t>
+  </si>
+  <si>
+    <t>polygons</t>
+  </si>
+  <si>
+    <t>protocols</t>
+  </si>
+  <si>
+    <t>samples</t>
+  </si>
+  <si>
+    <t>sites</t>
+  </si>
+  <si>
+    <t>contactID</t>
+  </si>
+  <si>
+    <t>instrumentID</t>
+  </si>
+  <si>
+    <t>datEmpty.organizations.__organizationID</t>
+  </si>
+  <si>
+    <t>datEmpty.measures.__measureRepID</t>
+  </si>
+  <si>
+    <t>datEmpty.contacts.__contactID</t>
+  </si>
+  <si>
+    <t>datEmpty.instruments.__instrumentID</t>
+  </si>
+  <si>
+    <t>polygonID</t>
+  </si>
+  <si>
+    <t>protocolID</t>
+  </si>
+  <si>
+    <t>datEmpty.protocols.__protocolID</t>
+  </si>
+  <si>
+    <t>datEmpty.polygons.__polygonID</t>
+  </si>
+  <si>
+    <t>sampleID</t>
+  </si>
+  <si>
+    <t>datEmpty.samples.__sampleID</t>
+  </si>
+  <si>
+    <t>datEmpty.sites.__siteID</t>
   </si>
 </sst>
 </file>
@@ -152,13 +209,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -473,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -495,79 +553,158 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-    </row>
+      <c r="B2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C16" t="s">
         <v>13</v>
       </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" t="s">
-        <v>8</v>
+      <c r="C23" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Linking to get organizationID
</commit_message>
<xml_diff>
--- a/data/odm_v2/odm_v1_to_v2_id_code.xlsx
+++ b/data/odm_v2/odm_v1_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/odm_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE629A60-1A16-E541-B1FF-BBCAA21A3C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C1888B-6AC7-154E-89E4-2D797D0C439E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>measures</t>
   </si>
@@ -95,70 +95,73 @@
     <t>organizationID</t>
   </si>
   <si>
+    <t>contacts</t>
+  </si>
+  <si>
+    <t>instruments</t>
+  </si>
+  <si>
+    <t>organizations</t>
+  </si>
+  <si>
+    <t>polygons</t>
+  </si>
+  <si>
+    <t>protocols</t>
+  </si>
+  <si>
+    <t>samples</t>
+  </si>
+  <si>
+    <t>sites</t>
+  </si>
+  <si>
+    <t>contactID</t>
+  </si>
+  <si>
+    <t>instrumentID</t>
+  </si>
+  <si>
+    <t>datEmpty.organizations.__organizationID</t>
+  </si>
+  <si>
+    <t>datEmpty.measures.__measureRepID</t>
+  </si>
+  <si>
+    <t>datEmpty.contacts.__contactID</t>
+  </si>
+  <si>
+    <t>datEmpty.instruments.__instrumentID</t>
+  </si>
+  <si>
+    <t>polygonID</t>
+  </si>
+  <si>
+    <t>protocolID</t>
+  </si>
+  <si>
+    <t>datEmpty.protocols.__protocolID</t>
+  </si>
+  <si>
+    <t>datEmpty.polygons.__polygonID</t>
+  </si>
+  <si>
+    <t>sampleID</t>
+  </si>
+  <si>
+    <t>datEmpty.samples.__sampleID</t>
+  </si>
+  <si>
+    <t>datEmpty.sites.__siteID</t>
+  </si>
+  <si>
+    <t>if fn.sourceclass in ["CovidPublicHealthData", "SiteMeasure"]:
+    target = dat.contacts.get_first_linked_value("organizationID", linkage_path={"source_slot":"contactID", "target_slot":"contactID"})
+else:
+    target = dat.measures.__organizationID</t>
+  </si>
+  <si>
     <t>dat.contacts.get_first_linked_value("organizationID", linkage_path={"source_slot":"contactID", "target_slot":"contactID"})</t>
-  </si>
-  <si>
-    <t>dat.measures.__organizationID</t>
-  </si>
-  <si>
-    <t>contacts</t>
-  </si>
-  <si>
-    <t>instruments</t>
-  </si>
-  <si>
-    <t>organizations</t>
-  </si>
-  <si>
-    <t>polygons</t>
-  </si>
-  <si>
-    <t>protocols</t>
-  </si>
-  <si>
-    <t>samples</t>
-  </si>
-  <si>
-    <t>sites</t>
-  </si>
-  <si>
-    <t>contactID</t>
-  </si>
-  <si>
-    <t>instrumentID</t>
-  </si>
-  <si>
-    <t>datEmpty.organizations.__organizationID</t>
-  </si>
-  <si>
-    <t>datEmpty.measures.__measureRepID</t>
-  </si>
-  <si>
-    <t>datEmpty.contacts.__contactID</t>
-  </si>
-  <si>
-    <t>datEmpty.instruments.__instrumentID</t>
-  </si>
-  <si>
-    <t>polygonID</t>
-  </si>
-  <si>
-    <t>protocolID</t>
-  </si>
-  <si>
-    <t>datEmpty.protocols.__protocolID</t>
-  </si>
-  <si>
-    <t>datEmpty.polygons.__polygonID</t>
-  </si>
-  <si>
-    <t>sampleID</t>
-  </si>
-  <si>
-    <t>datEmpty.samples.__sampleID</t>
-  </si>
-  <si>
-    <t>datEmpty.sites.__siteID</t>
   </si>
 </sst>
 </file>
@@ -209,14 +212,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -553,30 +555,28 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+    </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
@@ -585,7 +585,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -609,44 +609,41 @@
       <c r="B8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>18</v>
+      <c r="C8" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -687,24 +684,35 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" t="s">
         <v>37</v>
-      </c>
-      <c r="C21" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" t="s">
-        <v>14</v>
-      </c>
-      <c r="C23" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>